<commit_message>
Draw DexArm base footprint on 2D work-area boards
Adds a subtle, non-interactive outline of the DexArm base to the shared 2D
plate used by the Write&Draw, Laser and Control boards. Rebuilt and disposed
alongside the work area; labelled via i18n (EN/zh-CN/zh-TW).

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/web/i18n.xlsx
+++ b/web/i18n.xlsx
@@ -383,7 +383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K366"/>
+  <dimension ref="A1:K367"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -12608,9 +12608,20 @@
         <v>立即下载最新版 Rotrics Studio？</v>
       </c>
     </row>
+    <row r="367">
+      <c r="A367" t="str">
+        <v>DexArm Base</v>
+      </c>
+      <c r="B367" t="str">
+        <v>机械臂底座</v>
+      </c>
+      <c r="J367" t="str">
+        <v>機械臂底座</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K366"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K367"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>